<commit_message>
Add interactive sankey and HTML report output
</commit_message>
<xml_diff>
--- a/output/tables/enemdu_2025_ingreso_hogar_summary.xlsx
+++ b/output/tables/enemdu_2025_ingreso_hogar_summary.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t xml:space="preserve">scope</t>
   </si>
@@ -36,7 +36,7 @@
     <t xml:space="preserve">unweighted_median_income</t>
   </si>
   <si>
-    <t xml:space="preserve">households_with_missing_ingpc</t>
+    <t xml:space="preserve">households_excluded</t>
   </si>
   <si>
     <t xml:space="preserve">weighted_share_complete</t>
@@ -48,6 +48,12 @@
     <t xml:space="preserve">hh_income_total_from_ingpc</t>
   </si>
   <si>
+    <t xml:space="preserve">complete_labor_income_households</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hh_income_sum_ingrl</t>
+  </si>
+  <si>
     <t xml:space="preserve">item</t>
   </si>
   <si>
@@ -78,10 +84,22 @@
     <t xml:space="preserve">Household total income = ingpc * household size.</t>
   </si>
   <si>
+    <t xml:space="preserve">alternative_household_income_definition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alternative check: household labor income = sum of person-level ingrl within id_hogar.</t>
+  </si>
+  <si>
     <t xml:space="preserve">complete_income_rule</t>
   </si>
   <si>
     <t xml:space="preserve">Complete-income households require non-missing ingpc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">complete_labor_income_rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complete labor-income households exclude households where any person has ingrl = 999999; ingrl = -1 is kept as a valid labeled value.</t>
   </si>
   <si>
     <t xml:space="preserve">enighur_consistency_note</t>
@@ -474,6 +492,35 @@
         <v>0.993187536957529</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="n">
+        <v>104397</v>
+      </c>
+      <c r="D3" t="n">
+        <v>697.132083219587</v>
+      </c>
+      <c r="E3" t="n">
+        <v>490</v>
+      </c>
+      <c r="F3" t="n">
+        <v>777.325881011907</v>
+      </c>
+      <c r="G3" t="n">
+        <v>520</v>
+      </c>
+      <c r="H3" t="n">
+        <v>341</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.997274232659811</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -487,58 +534,74 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>